<commit_message>
Integración ERP/base de datos: sábana de gestiones exportable/sincronizable
- kobra/integracion.py: sábana con tipificación completa (Pago/Arreglo de pago/
  Informado/No contactado/Fallecido/…), fechas, montos, notas, tipo_gestor;
  exporta JSON/CSV/Excel, envía por API REST y sincroniza a cualquier base SQL
  (SQLAlchemy). Mapeo de campos opcional.
- registro/gestor_ia/generate_gestiones: esquema extendido con la tipificación
  y datos (fecha compromiso/pago, monto acordado, cuotas, descuento, notas).
- Dashboard: pestaña 'Integración ERP' (vista previa + descarga + envío/sync).
- Config: ERP_API_URL/API_KEY/DB_URL. requirements: sqlalchemy. Tests 42/42.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KGnVQvVgKrpMBAH6ciJfTu
</commit_message>
<xml_diff>
--- a/outputs/kobra_analitica_gestion.xlsx
+++ b/outputs/kobra_analitica_gestion.xlsx
@@ -47,88 +47,88 @@
     <t>tasa_recupero</t>
   </si>
   <si>
+    <t>IA02</t>
+  </si>
+  <si>
     <t>IA01</t>
   </si>
   <si>
-    <t>IA02</t>
-  </si>
-  <si>
     <t>G04</t>
   </si>
   <si>
+    <t>G03</t>
+  </si>
+  <si>
+    <t>G12</t>
+  </si>
+  <si>
+    <t>G09</t>
+  </si>
+  <si>
+    <t>G08</t>
+  </si>
+  <si>
+    <t>G07</t>
+  </si>
+  <si>
     <t>G11</t>
   </si>
   <si>
+    <t>G01</t>
+  </si>
+  <si>
+    <t>G10</t>
+  </si>
+  <si>
+    <t>G05</t>
+  </si>
+  <si>
+    <t>G06</t>
+  </si>
+  <si>
     <t>G02</t>
   </si>
   <si>
-    <t>G09</t>
-  </si>
-  <si>
-    <t>G03</t>
-  </si>
-  <si>
-    <t>G10</t>
-  </si>
-  <si>
-    <t>G12</t>
-  </si>
-  <si>
-    <t>G01</t>
-  </si>
-  <si>
-    <t>G08</t>
-  </si>
-  <si>
-    <t>G07</t>
-  </si>
-  <si>
-    <t>G06</t>
-  </si>
-  <si>
-    <t>G05</t>
+    <t>Gestor IA02</t>
   </si>
   <si>
     <t>Gestor IA01</t>
   </si>
   <si>
-    <t>Gestor IA02</t>
-  </si>
-  <si>
     <t>Gestor 04</t>
   </si>
   <si>
+    <t>Gestor 03</t>
+  </si>
+  <si>
+    <t>Gestor 12</t>
+  </si>
+  <si>
+    <t>Gestor 09</t>
+  </si>
+  <si>
+    <t>Gestor 08</t>
+  </si>
+  <si>
+    <t>Gestor 07</t>
+  </si>
+  <si>
     <t>Gestor 11</t>
   </si>
   <si>
+    <t>Gestor 01</t>
+  </si>
+  <si>
+    <t>Gestor 10</t>
+  </si>
+  <si>
+    <t>Gestor 05</t>
+  </si>
+  <si>
+    <t>Gestor 06</t>
+  </si>
+  <si>
     <t>Gestor 02</t>
-  </si>
-  <si>
-    <t>Gestor 09</t>
-  </si>
-  <si>
-    <t>Gestor 03</t>
-  </si>
-  <si>
-    <t>Gestor 10</t>
-  </si>
-  <si>
-    <t>Gestor 12</t>
-  </si>
-  <si>
-    <t>Gestor 01</t>
-  </si>
-  <si>
-    <t>Gestor 08</t>
-  </si>
-  <si>
-    <t>Gestor 07</t>
-  </si>
-  <si>
-    <t>Gestor 06</t>
-  </si>
-  <si>
-    <t>Gestor 05</t>
   </si>
   <si>
     <t>calidad_inicial</t>
@@ -611,22 +611,22 @@
         <v>840</v>
       </c>
       <c r="D2">
-        <v>84.142</v>
+        <v>83.973</v>
       </c>
       <c r="E2">
-        <v>70588327</v>
+        <v>69248494</v>
       </c>
       <c r="F2">
-        <v>145243350</v>
+        <v>129478740</v>
       </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2">
-        <v>0.801</v>
+        <v>0.774</v>
       </c>
       <c r="I2">
-        <v>0.486</v>
+        <v>0.535</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -640,22 +640,22 @@
         <v>840</v>
       </c>
       <c r="D3">
-        <v>84.074</v>
+        <v>83.84699999999999</v>
       </c>
       <c r="E3">
-        <v>58070851</v>
+        <v>55552435</v>
       </c>
       <c r="F3">
-        <v>125395480</v>
+        <v>119757140</v>
       </c>
       <c r="G3" t="b">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>0.795</v>
+        <v>0.758</v>
       </c>
       <c r="I3">
-        <v>0.463</v>
+        <v>0.464</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -669,22 +669,22 @@
         <v>485</v>
       </c>
       <c r="D4">
-        <v>74.886</v>
+        <v>75.39400000000001</v>
       </c>
       <c r="E4">
-        <v>35017013</v>
+        <v>37666889</v>
       </c>
       <c r="F4">
-        <v>96027400</v>
+        <v>76705570</v>
       </c>
       <c r="G4" t="b">
         <v>1</v>
       </c>
       <c r="H4">
-        <v>0.711</v>
+        <v>0.755</v>
       </c>
       <c r="I4">
-        <v>0.365</v>
+        <v>0.491</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -695,25 +695,25 @@
         <v>26</v>
       </c>
       <c r="C5">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D5">
-        <v>78.732</v>
+        <v>73.22</v>
       </c>
       <c r="E5">
-        <v>34339300</v>
+        <v>35475125</v>
       </c>
       <c r="F5">
-        <v>71991100</v>
+        <v>75917050</v>
       </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
       <c r="H5">
-        <v>0.751</v>
+        <v>0.733</v>
       </c>
       <c r="I5">
-        <v>0.477</v>
+        <v>0.467</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -724,25 +724,25 @@
         <v>27</v>
       </c>
       <c r="C6">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D6">
-        <v>52.532</v>
+        <v>75.14</v>
       </c>
       <c r="E6">
-        <v>34101867</v>
+        <v>34093167</v>
       </c>
       <c r="F6">
-        <v>73592050</v>
+        <v>68232610</v>
       </c>
       <c r="G6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>0.532</v>
+        <v>0.754</v>
       </c>
       <c r="I6">
-        <v>0.463</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -756,22 +756,22 @@
         <v>471</v>
       </c>
       <c r="D7">
-        <v>67.666</v>
+        <v>67.13800000000001</v>
       </c>
       <c r="E7">
-        <v>33804167</v>
+        <v>31633466</v>
       </c>
       <c r="F7">
-        <v>83215730</v>
+        <v>68861150</v>
       </c>
       <c r="G7" t="b">
         <v>1</v>
       </c>
       <c r="H7">
-        <v>0.675</v>
+        <v>0.605</v>
       </c>
       <c r="I7">
-        <v>0.406</v>
+        <v>0.459</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -782,25 +782,25 @@
         <v>29</v>
       </c>
       <c r="C8">
-        <v>468</v>
+        <v>449</v>
       </c>
       <c r="D8">
-        <v>73.217</v>
+        <v>64.45699999999999</v>
       </c>
       <c r="E8">
-        <v>33394337</v>
+        <v>31580546</v>
       </c>
       <c r="F8">
-        <v>65175150</v>
+        <v>87475510</v>
       </c>
       <c r="G8" t="b">
         <v>1</v>
       </c>
       <c r="H8">
-        <v>0.701</v>
+        <v>0.619</v>
       </c>
       <c r="I8">
-        <v>0.512</v>
+        <v>0.361</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -811,25 +811,25 @@
         <v>30</v>
       </c>
       <c r="C9">
-        <v>451</v>
+        <v>477</v>
       </c>
       <c r="D9">
-        <v>62.257</v>
+        <v>69.559</v>
       </c>
       <c r="E9">
-        <v>30435154</v>
+        <v>30896368</v>
       </c>
       <c r="F9">
-        <v>76741760</v>
+        <v>63145260</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
       </c>
       <c r="H9">
-        <v>0.61</v>
+        <v>0.675</v>
       </c>
       <c r="I9">
-        <v>0.397</v>
+        <v>0.489</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -840,25 +840,25 @@
         <v>31</v>
       </c>
       <c r="C10">
-        <v>460</v>
+        <v>470</v>
       </c>
       <c r="D10">
-        <v>75.142</v>
+        <v>79.167</v>
       </c>
       <c r="E10">
-        <v>29905289</v>
+        <v>30775207</v>
       </c>
       <c r="F10">
-        <v>73518440</v>
+        <v>68493150</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
       </c>
       <c r="H10">
-        <v>0.728</v>
+        <v>0.745</v>
       </c>
       <c r="I10">
-        <v>0.407</v>
+        <v>0.449</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -872,22 +872,22 @@
         <v>472</v>
       </c>
       <c r="D11">
-        <v>64.395</v>
+        <v>63.824</v>
       </c>
       <c r="E11">
-        <v>29190869</v>
+        <v>28015532</v>
       </c>
       <c r="F11">
-        <v>75235140</v>
+        <v>74979340</v>
       </c>
       <c r="G11" t="b">
         <v>0</v>
       </c>
       <c r="H11">
-        <v>0.633</v>
+        <v>0.657</v>
       </c>
       <c r="I11">
-        <v>0.388</v>
+        <v>0.374</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -898,25 +898,25 @@
         <v>33</v>
       </c>
       <c r="C12">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="D12">
-        <v>64.51000000000001</v>
+        <v>61.555</v>
       </c>
       <c r="E12">
-        <v>28403371</v>
+        <v>25146877</v>
       </c>
       <c r="F12">
-        <v>65243820</v>
+        <v>66876290</v>
       </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12">
-        <v>0.639</v>
+        <v>0.601</v>
       </c>
       <c r="I12">
-        <v>0.435</v>
+        <v>0.376</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -927,25 +927,25 @@
         <v>34</v>
       </c>
       <c r="C13">
-        <v>477</v>
+        <v>456</v>
       </c>
       <c r="D13">
-        <v>69.352</v>
+        <v>50.071</v>
       </c>
       <c r="E13">
-        <v>28317702</v>
+        <v>22196467</v>
       </c>
       <c r="F13">
-        <v>74809270</v>
+        <v>69382250</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
       </c>
       <c r="H13">
-        <v>0.648</v>
+        <v>0.531</v>
       </c>
       <c r="I13">
-        <v>0.379</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -959,22 +959,22 @@
         <v>461</v>
       </c>
       <c r="D14">
-        <v>54.214</v>
+        <v>53.653</v>
       </c>
       <c r="E14">
-        <v>21102721</v>
+        <v>21451311</v>
       </c>
       <c r="F14">
-        <v>71423870</v>
+        <v>59492300</v>
       </c>
       <c r="G14" t="b">
         <v>1</v>
       </c>
       <c r="H14">
-        <v>0.529</v>
+        <v>0.584</v>
       </c>
       <c r="I14">
-        <v>0.295</v>
+        <v>0.361</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -985,25 +985,25 @@
         <v>36</v>
       </c>
       <c r="C15">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="D15">
-        <v>50.884</v>
+        <v>52.775</v>
       </c>
       <c r="E15">
-        <v>19553068</v>
+        <v>19181382</v>
       </c>
       <c r="F15">
-        <v>60246360</v>
+        <v>51606410</v>
       </c>
       <c r="G15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>0.533</v>
+        <v>0.575</v>
       </c>
       <c r="I15">
-        <v>0.325</v>
+        <v>0.372</v>
       </c>
     </row>
   </sheetData>
@@ -1047,321 +1047,321 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>43.5</v>
+        <v>43.1</v>
       </c>
       <c r="E2">
-        <v>58.2</v>
+        <v>57</v>
       </c>
       <c r="F2">
-        <v>14.8</v>
+        <v>13.9</v>
       </c>
       <c r="G2">
         <v>0.452</v>
       </c>
       <c r="H2">
-        <v>0.573</v>
+        <v>0.581</v>
       </c>
       <c r="I2">
-        <v>0.121</v>
+        <v>0.129</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>62.7</v>
+        <v>68.7</v>
       </c>
       <c r="E3">
-        <v>74.5</v>
+        <v>82.2</v>
       </c>
       <c r="F3">
-        <v>11.8</v>
+        <v>13.5</v>
       </c>
       <c r="G3">
-        <v>0.622</v>
+        <v>0.742</v>
       </c>
       <c r="H3">
-        <v>0.672</v>
+        <v>0.789</v>
       </c>
       <c r="I3">
-        <v>0.05</v>
+        <v>0.046</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>62.1</v>
+        <v>54.2</v>
       </c>
       <c r="E4">
-        <v>73.90000000000001</v>
+        <v>67</v>
       </c>
       <c r="F4">
-        <v>11.8</v>
+        <v>12.8</v>
       </c>
       <c r="G4">
-        <v>0.649</v>
+        <v>0.552</v>
       </c>
       <c r="H4">
-        <v>0.695</v>
+        <v>0.669</v>
       </c>
       <c r="I4">
-        <v>0.046</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>71.90000000000001</v>
+        <v>60.8</v>
       </c>
       <c r="E5">
-        <v>83.7</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="F5">
-        <v>11.7</v>
+        <v>12.6</v>
       </c>
       <c r="G5">
-        <v>0.713</v>
+        <v>0.582</v>
       </c>
       <c r="H5">
-        <v>0.75</v>
+        <v>0.703</v>
       </c>
       <c r="I5">
-        <v>0.037</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>69.3</v>
+        <v>62.9</v>
       </c>
       <c r="E6">
-        <v>80.90000000000001</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="F6">
-        <v>11.6</v>
+        <v>12.5</v>
       </c>
       <c r="G6">
-        <v>0.6879999999999999</v>
+        <v>0.647</v>
       </c>
       <c r="H6">
-        <v>0.764</v>
+        <v>0.723</v>
       </c>
       <c r="I6">
-        <v>0.077</v>
+        <v>0.076</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>68.09999999999999</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="E7">
-        <v>79.59999999999999</v>
+        <v>80</v>
       </c>
       <c r="F7">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="G7">
         <v>0.732</v>
       </c>
       <c r="H7">
-        <v>0.73</v>
+        <v>0.795</v>
       </c>
       <c r="I7">
-        <v>-0.002</v>
+        <v>0.063</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>55.3</v>
+        <v>70.2</v>
       </c>
       <c r="E8">
-        <v>66.7</v>
+        <v>81.5</v>
       </c>
       <c r="F8">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="G8">
-        <v>0.526</v>
+        <v>0.752</v>
       </c>
       <c r="H8">
-        <v>0.661</v>
+        <v>0.782</v>
       </c>
       <c r="I8">
-        <v>0.135</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>58.6</v>
+        <v>48.9</v>
       </c>
       <c r="E9">
-        <v>69.40000000000001</v>
+        <v>60.2</v>
       </c>
       <c r="F9">
-        <v>10.8</v>
+        <v>11.3</v>
       </c>
       <c r="G9">
-        <v>0.598</v>
+        <v>0.492</v>
       </c>
       <c r="H9">
-        <v>0.6899999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="I9">
-        <v>0.091</v>
+        <v>0.185</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
       </c>
       <c r="D10">
-        <v>70.59999999999999</v>
+        <v>59.7</v>
       </c>
       <c r="E10">
-        <v>81.2</v>
+        <v>70</v>
       </c>
       <c r="F10">
-        <v>10.7</v>
+        <v>10.2</v>
       </c>
       <c r="G10">
-        <v>0.6860000000000001</v>
+        <v>0.646</v>
       </c>
       <c r="H10">
-        <v>0.805</v>
+        <v>0.698</v>
       </c>
       <c r="I10">
-        <v>0.118</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
       </c>
       <c r="D11">
-        <v>51</v>
+        <v>72.8</v>
       </c>
       <c r="E11">
-        <v>59.1</v>
+        <v>83</v>
       </c>
       <c r="F11">
-        <v>8.199999999999999</v>
+        <v>10.2</v>
       </c>
       <c r="G11">
-        <v>0.523</v>
+        <v>0.583</v>
       </c>
       <c r="H11">
-        <v>0.5649999999999999</v>
+        <v>0.757</v>
       </c>
       <c r="I11">
-        <v>0.041</v>
+        <v>0.175</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C12" t="b">
         <v>0</v>
       </c>
       <c r="D12">
-        <v>53</v>
+        <v>52.1</v>
       </c>
       <c r="E12">
-        <v>53.1</v>
+        <v>52.7</v>
       </c>
       <c r="F12">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="G12">
-        <v>0.488</v>
+        <v>0.551</v>
       </c>
       <c r="H12">
-        <v>0.586</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="I12">
-        <v>0.098</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1375,22 +1375,22 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>65.7</v>
+        <v>63.4</v>
       </c>
       <c r="E13">
-        <v>64.2</v>
+        <v>62.8</v>
       </c>
       <c r="F13">
-        <v>-1.6</v>
+        <v>-0.6</v>
       </c>
       <c r="G13">
-        <v>0.617</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="H13">
-        <v>0.6830000000000001</v>
+        <v>0.634</v>
       </c>
       <c r="I13">
-        <v>0.066</v>
+        <v>-0.05</v>
       </c>
     </row>
   </sheetData>
@@ -1437,22 +1437,22 @@
         <v>511</v>
       </c>
       <c r="C2">
-        <v>60.861</v>
+        <v>60.633</v>
       </c>
       <c r="D2">
-        <v>-0.048</v>
+        <v>-0.061</v>
       </c>
       <c r="E2">
-        <v>43821999</v>
+        <v>27669758</v>
       </c>
       <c r="F2">
-        <v>94466210</v>
+        <v>70929990</v>
       </c>
       <c r="G2">
-        <v>0.601</v>
+        <v>0.626</v>
       </c>
       <c r="H2">
-        <v>0.464</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1463,22 +1463,22 @@
         <v>502</v>
       </c>
       <c r="C3">
-        <v>60.773</v>
+        <v>60.487</v>
       </c>
       <c r="D3">
-        <v>-0.081</v>
+        <v>-0.075</v>
       </c>
       <c r="E3">
-        <v>33133394</v>
+        <v>29746874</v>
       </c>
       <c r="F3">
-        <v>87896090</v>
+        <v>77458350</v>
       </c>
       <c r="G3">
-        <v>0.594</v>
+        <v>0.629</v>
       </c>
       <c r="H3">
-        <v>0.377</v>
+        <v>0.384</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1489,22 +1489,22 @@
         <v>515</v>
       </c>
       <c r="C4">
-        <v>61.62</v>
+        <v>60.448</v>
       </c>
       <c r="D4">
-        <v>-0.08699999999999999</v>
+        <v>-0.073</v>
       </c>
       <c r="E4">
-        <v>30985799</v>
+        <v>26768785</v>
       </c>
       <c r="F4">
-        <v>79875320</v>
+        <v>60371900</v>
       </c>
       <c r="G4">
-        <v>0.633</v>
+        <v>0.606</v>
       </c>
       <c r="H4">
-        <v>0.388</v>
+        <v>0.443</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1515,22 +1515,22 @@
         <v>503</v>
       </c>
       <c r="C5">
-        <v>61.422</v>
+        <v>61.847</v>
       </c>
       <c r="D5">
-        <v>-0.08500000000000001</v>
+        <v>-0.033</v>
       </c>
       <c r="E5">
-        <v>41503271</v>
+        <v>34796900</v>
       </c>
       <c r="F5">
-        <v>96943360</v>
+        <v>80216640</v>
       </c>
       <c r="G5">
-        <v>0.64</v>
+        <v>0.646</v>
       </c>
       <c r="H5">
-        <v>0.428</v>
+        <v>0.434</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1541,22 +1541,22 @@
         <v>515</v>
       </c>
       <c r="C6">
-        <v>63.95</v>
+        <v>63.454</v>
       </c>
       <c r="D6">
-        <v>-0.064</v>
+        <v>-0.03</v>
       </c>
       <c r="E6">
-        <v>24281194</v>
+        <v>30139458</v>
       </c>
       <c r="F6">
-        <v>73881600</v>
+        <v>79615060</v>
       </c>
       <c r="G6">
-        <v>0.627</v>
+        <v>0.633</v>
       </c>
       <c r="H6">
-        <v>0.329</v>
+        <v>0.379</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1567,22 +1567,22 @@
         <v>508</v>
       </c>
       <c r="C7">
-        <v>66.19499999999999</v>
+        <v>66.38500000000001</v>
       </c>
       <c r="D7">
-        <v>-0.058</v>
+        <v>-0.045</v>
       </c>
       <c r="E7">
-        <v>30268936</v>
+        <v>23433111</v>
       </c>
       <c r="F7">
-        <v>80156620</v>
+        <v>72856850</v>
       </c>
       <c r="G7">
-        <v>0.614</v>
+        <v>0.618</v>
       </c>
       <c r="H7">
-        <v>0.378</v>
+        <v>0.322</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1593,22 +1593,22 @@
         <v>840</v>
       </c>
       <c r="C8">
-        <v>74.38</v>
+        <v>74.503</v>
       </c>
       <c r="D8">
-        <v>-0.01</v>
+        <v>0.001</v>
       </c>
       <c r="E8">
-        <v>58253021</v>
+        <v>64433898</v>
       </c>
       <c r="F8">
-        <v>131524770</v>
+        <v>142265630</v>
       </c>
       <c r="G8">
-        <v>0.679</v>
+        <v>0.696</v>
       </c>
       <c r="H8">
-        <v>0.443</v>
+        <v>0.453</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1619,22 +1619,22 @@
         <v>842</v>
       </c>
       <c r="C9">
-        <v>75.276</v>
+        <v>74.812</v>
       </c>
       <c r="D9">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="E9">
-        <v>45622776</v>
+        <v>60455407</v>
       </c>
       <c r="F9">
-        <v>115094610</v>
+        <v>125160080</v>
       </c>
       <c r="G9">
-        <v>0.736</v>
+        <v>0.728</v>
       </c>
       <c r="H9">
-        <v>0.396</v>
+        <v>0.483</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1645,22 +1645,22 @@
         <v>833</v>
       </c>
       <c r="C10">
-        <v>75.571</v>
+        <v>75.06100000000001</v>
       </c>
       <c r="D10">
-        <v>0.005</v>
+        <v>-0.021</v>
       </c>
       <c r="E10">
-        <v>64302657</v>
+        <v>56120573</v>
       </c>
       <c r="F10">
-        <v>131721500</v>
+        <v>123916800</v>
       </c>
       <c r="G10">
-        <v>0.726</v>
+        <v>0.699</v>
       </c>
       <c r="H10">
-        <v>0.488</v>
+        <v>0.453</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1671,22 +1671,22 @@
         <v>840</v>
       </c>
       <c r="C11">
-        <v>75.971</v>
+        <v>76.61499999999999</v>
       </c>
       <c r="D11">
-        <v>-0.006</v>
+        <v>-0.011</v>
       </c>
       <c r="E11">
-        <v>57509386</v>
+        <v>66020284</v>
       </c>
       <c r="F11">
-        <v>133092280</v>
+        <v>128016570</v>
       </c>
       <c r="G11">
-        <v>0.736</v>
+        <v>0.744</v>
       </c>
       <c r="H11">
-        <v>0.432</v>
+        <v>0.516</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1697,22 +1697,22 @@
         <v>850</v>
       </c>
       <c r="C12">
-        <v>76.14700000000001</v>
+        <v>75.938</v>
       </c>
       <c r="D12">
-        <v>-0.011</v>
+        <v>-0.008</v>
       </c>
       <c r="E12">
-        <v>56541603</v>
+        <v>53328218</v>
       </c>
       <c r="F12">
-        <v>133206560</v>
+        <v>119594900</v>
       </c>
       <c r="G12">
-        <v>0.729</v>
+        <v>0.725</v>
       </c>
       <c r="H12">
-        <v>0.424</v>
+        <v>0.446</v>
       </c>
     </row>
   </sheetData>
@@ -1762,28 +1762,28 @@
         <v>59</v>
       </c>
       <c r="B2">
-        <v>2005</v>
+        <v>2100</v>
       </c>
       <c r="C2">
-        <v>69.99299999999999</v>
+        <v>69.667</v>
       </c>
       <c r="D2">
-        <v>0.189</v>
+        <v>0.199</v>
       </c>
       <c r="E2">
-        <v>3.479</v>
+        <v>3.501</v>
       </c>
       <c r="F2">
-        <v>159756257</v>
+        <v>176079513</v>
       </c>
       <c r="G2">
-        <v>330376450</v>
+        <v>330563200</v>
       </c>
       <c r="H2">
-        <v>0.755</v>
+        <v>0.76</v>
       </c>
       <c r="I2">
-        <v>0.484</v>
+        <v>0.533</v>
       </c>
       <c r="J2" t="s">
         <v>64</v>
@@ -1794,28 +1794,28 @@
         <v>60</v>
       </c>
       <c r="B3">
-        <v>643</v>
+        <v>663</v>
       </c>
       <c r="C3">
-        <v>69.13500000000001</v>
+        <v>70.18600000000001</v>
       </c>
       <c r="D3">
-        <v>-0.318</v>
+        <v>-0.317</v>
       </c>
       <c r="E3">
-        <v>3.439</v>
+        <v>3.466</v>
       </c>
       <c r="F3">
-        <v>16390957</v>
+        <v>22121212</v>
       </c>
       <c r="G3">
-        <v>83897890</v>
+        <v>95315280</v>
       </c>
       <c r="H3">
-        <v>0.468</v>
+        <v>0.504</v>
       </c>
       <c r="I3">
-        <v>0.195</v>
+        <v>0.232</v>
       </c>
       <c r="J3" t="s">
         <v>65</v>
@@ -1826,28 +1826,28 @@
         <v>61</v>
       </c>
       <c r="B4">
-        <v>1861</v>
+        <v>1771</v>
       </c>
       <c r="C4">
-        <v>69.949</v>
+        <v>69.489</v>
       </c>
       <c r="D4">
         <v>0.101</v>
       </c>
       <c r="E4">
-        <v>3.485</v>
+        <v>3.497</v>
       </c>
       <c r="F4">
-        <v>130455786</v>
+        <v>104473017</v>
       </c>
       <c r="G4">
-        <v>280704560</v>
+        <v>228459790</v>
       </c>
       <c r="H4">
-        <v>0.733</v>
+        <v>0.725</v>
       </c>
       <c r="I4">
-        <v>0.465</v>
+        <v>0.457</v>
       </c>
       <c r="J4" t="s">
         <v>64</v>
@@ -1858,28 +1858,28 @@
         <v>62</v>
       </c>
       <c r="B5">
-        <v>1163</v>
+        <v>1169</v>
       </c>
       <c r="C5">
-        <v>70.538</v>
+        <v>70.19499999999999</v>
       </c>
       <c r="D5">
-        <v>-0.167</v>
+        <v>-0.157</v>
       </c>
       <c r="E5">
-        <v>3.5</v>
+        <v>3.506</v>
       </c>
       <c r="F5">
-        <v>76657465</v>
+        <v>74071299</v>
       </c>
       <c r="G5">
-        <v>184543420</v>
+        <v>162093480</v>
       </c>
       <c r="H5">
-        <v>0.669</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="I5">
-        <v>0.415</v>
+        <v>0.457</v>
       </c>
       <c r="J5" t="s">
         <v>66</v>
@@ -1890,28 +1890,28 @@
         <v>63</v>
       </c>
       <c r="B6">
-        <v>1587</v>
+        <v>1556</v>
       </c>
       <c r="C6">
-        <v>70.039</v>
+        <v>70.07599999999999</v>
       </c>
       <c r="D6">
-        <v>-0.246</v>
+        <v>-0.25</v>
       </c>
       <c r="E6">
-        <v>3.491</v>
+        <v>3.511</v>
       </c>
       <c r="F6">
-        <v>102963571</v>
+        <v>96168225</v>
       </c>
       <c r="G6">
-        <v>278336600</v>
+        <v>263971020</v>
       </c>
       <c r="H6">
-        <v>0.607</v>
+        <v>0.593</v>
       </c>
       <c r="I6">
-        <v>0.37</v>
+        <v>0.364</v>
       </c>
       <c r="J6" t="s">
         <v>67</v>
@@ -1964,28 +1964,28 @@
         <v>69</v>
       </c>
       <c r="B2">
-        <v>780</v>
+        <v>749</v>
       </c>
       <c r="C2">
-        <v>70.233</v>
+        <v>70.068</v>
       </c>
       <c r="D2">
-        <v>-0.056</v>
+        <v>-0.044</v>
       </c>
       <c r="E2">
-        <v>3.437</v>
+        <v>3.453</v>
       </c>
       <c r="F2">
-        <v>289425800</v>
+        <v>277602721</v>
       </c>
       <c r="G2">
-        <v>706338850</v>
+        <v>619859410</v>
       </c>
       <c r="H2">
-        <v>0.672</v>
+        <v>0.668</v>
       </c>
       <c r="I2">
-        <v>0.41</v>
+        <v>0.448</v>
       </c>
       <c r="J2" t="s">
         <v>72</v>
@@ -1996,31 +1996,31 @@
         <v>70</v>
       </c>
       <c r="B3">
-        <v>2054</v>
+        <v>2079</v>
       </c>
       <c r="C3">
-        <v>69.801</v>
+        <v>69.26300000000001</v>
       </c>
       <c r="D3">
-        <v>-0.033</v>
+        <v>-0.031</v>
       </c>
       <c r="E3">
-        <v>3.444</v>
+        <v>3.473</v>
       </c>
       <c r="F3">
-        <v>131801528</v>
+        <v>129193592</v>
       </c>
       <c r="G3">
-        <v>300703240</v>
+        <v>307640510</v>
       </c>
       <c r="H3">
-        <v>0.6820000000000001</v>
+        <v>0.68</v>
       </c>
       <c r="I3">
-        <v>0.438</v>
+        <v>0.42</v>
       </c>
       <c r="J3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2028,28 +2028,28 @@
         <v>71</v>
       </c>
       <c r="B4">
-        <v>4425</v>
+        <v>4431</v>
       </c>
       <c r="C4">
-        <v>70.057</v>
+        <v>70.078</v>
       </c>
       <c r="D4">
-        <v>-0.025</v>
+        <v>-0.019</v>
       </c>
       <c r="E4">
-        <v>3.509</v>
+        <v>3.521</v>
       </c>
       <c r="F4">
-        <v>64996708</v>
+        <v>66116953</v>
       </c>
       <c r="G4">
-        <v>150816830</v>
+        <v>152902850</v>
       </c>
       <c r="H4">
-        <v>0.677</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="I4">
-        <v>0.431</v>
+        <v>0.432</v>
       </c>
       <c r="J4" t="s">
         <v>72</v>

</xml_diff>